<commit_message>
feat: add dashboard, schedule, affective pages and associated API routes
</commit_message>
<xml_diff>
--- a/public/templates/sample_schedule.xlsx
+++ b/public/templates/sample_schedule.xlsx
@@ -494,7 +494,7 @@
         <v>ปฏิบัติ</v>
       </c>
       <c r="I3" t="str">
-        <v>อ.ชญารัตน์</v>
+        <v>อ.xxxx</v>
       </c>
     </row>
     <row r="4">
@@ -552,7 +552,7 @@
         <v>ทฤษฎี</v>
       </c>
       <c r="I5" t="str">
-        <v>อ.ศิริยา</v>
+        <v>อ.xxxx</v>
       </c>
     </row>
     <row r="6">
@@ -581,7 +581,7 @@
         <v>ปฏิบัติ</v>
       </c>
       <c r="I6" t="str">
-        <v>อ.จริญยา</v>
+        <v>อ.xxxx</v>
       </c>
     </row>
     <row r="7">
@@ -639,7 +639,7 @@
         <v>ปฏิบัติ</v>
       </c>
       <c r="I8" t="str">
-        <v>อ.วิโรจน์</v>
+        <v>อ.xxxx</v>
       </c>
     </row>
     <row r="9">
@@ -668,7 +668,7 @@
         <v>ทฤษฎี</v>
       </c>
       <c r="I9" t="str">
-        <v>Teacher John</v>
+        <v>Teacher xxx</v>
       </c>
     </row>
   </sheetData>

</xml_diff>